<commit_message>
feat: carga de planejado so de volume, valor opcional (migration 325); Pecas continua exigindo valor
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/modelo-carga-vendas-planejado.xlsx
+++ b/templates/modelo-carga-vendas-planejado.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Meta Vendas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meta Vendas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -654,6 +654,7 @@
       </c>
       <c r="F9" s="5" t="n"/>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
@@ -685,14 +686,14 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>quantidade  -&gt; quantidade planejada no mês. OPCIONAL para Transgrain/Acessórios (meta só por valor).</t>
+          <t>quantidade  -&gt; quantidade planejada no mês (volume). OPCIONAL só para Transgrain/Acessórios</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>valor       -&gt; valor planejado no mês em R$ (sempre obrigatório)</t>
+          <t>valor       -&gt; valor planejado no mês em R$. OPCIONAL (a meta é de volume); obrigatório só para Peças</t>
         </is>
       </c>
     </row>
@@ -703,10 +704,11 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Transgrain/Acessórios -&gt; meta só por VALOR, SEM gestão: quantidade e território opcionais; somam no card lateral do painel, por tipo. Peças usa a meta da coordenação Peças (Jenifer).</t>
+          <t>Transgrain/Acessórios -&gt; quantidade e território opcionais; somam no card lateral do painel, por tipo. Peças usa a meta da coordenação Peças (Jenifer), em valor.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: carga de planejado com volume obrigatorio (exceto Pecas); valor e %MB vazios assumem o cenario (migration 326)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/modelo-carga-vendas-planejado.xlsx
+++ b/templates/modelo-carga-vendas-planejado.xlsx
@@ -686,21 +686,21 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>quantidade  -&gt; quantidade planejada no mês (volume). OPCIONAL só para Transgrain/Acessórios</t>
+          <t>quantidade  -&gt; volume planejado no mês. OBRIGATÓRIO para tudo que não seja Peças</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>valor       -&gt; valor planejado no mês em R$. OPCIONAL (a meta é de volume); obrigatório só para Peças</t>
+          <t>valor       -&gt; valor planejado no mês em R$. Em branco, assume quantidade × FAT/un do cenário de planejamento. OBRIGATÓRIO só para Peças</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>%MB         -&gt; margem bruta % (OPCIONAL)</t>
+          <t>%MB         -&gt; margem bruta %. Em branco, assume a do cenário de planejamento (premissas e impostos do FAT)</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Transgrain/Acessórios -&gt; quantidade e território opcionais; somam no card lateral do painel, por tipo. Peças usa a meta da coordenação Peças (Jenifer), em valor.</t>
+          <t>Transgrain/Acessórios -&gt; território opcional; somam no card lateral do painel, por tipo. Peças usa a meta da coordenação Peças (Jenifer), em valor.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: meta do Painel acompanha o cenario e o FAT (migrations 327, 328, 329); %MB passa a MC1%
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/modelo-carga-vendas-planejado.xlsx
+++ b/templates/modelo-carga-vendas-planejado.xlsx
@@ -480,7 +480,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>%MB</t>
+          <t>MC1%</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>%MB         -&gt; margem bruta %. Em branco, assume a do cenário de planejamento (premissas e impostos do FAT)</t>
+          <t>MC1%         -&gt; MC1 %. Em branco, assume a do cenário de planejamento (premissas e impostos do FAT)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: importacao de Planejado nos formularios do cenario (Excel, so admin), lancamento sem centro de custo, FAT/CPX prevalecem sobre 08/04 e carga de planejado vendas com campos obrigatorios
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/modelo-carga-vendas-planejado.xlsx
+++ b/templates/modelo-carga-vendas-planejado.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -478,11 +478,6 @@
           <t>valor</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>MC1%</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -504,9 +499,6 @@
       <c r="E2" s="4" t="n">
         <v>78863.91</v>
       </c>
-      <c r="F2" s="5" t="n">
-        <v>0.477</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -528,9 +520,6 @@
       <c r="E3" s="4" t="n">
         <v>206460</v>
       </c>
-      <c r="F3" s="5" t="n">
-        <v>0.64</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -552,9 +541,6 @@
       <c r="E4" s="4" t="n">
         <v>79500</v>
       </c>
-      <c r="F4" s="5" t="n">
-        <v>0.477</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -565,14 +551,17 @@
       <c r="B5" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="C5" s="3" t="n"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>GO_MG SUL</t>
+        </is>
+      </c>
       <c r="D5" s="3" t="n">
         <v>50</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>31875</v>
       </c>
-      <c r="F5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -594,9 +583,6 @@
       <c r="E6" s="4" t="n">
         <v>15356</v>
       </c>
-      <c r="F6" s="5" t="n">
-        <v>0.481</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -618,9 +604,6 @@
       <c r="E7" s="4" t="n">
         <v>430000</v>
       </c>
-      <c r="F7" s="5" t="n">
-        <v>0.3</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -631,12 +614,17 @@
       <c r="B8" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="E8" s="4" t="n">
         <v>60000</v>
       </c>
-      <c r="F8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -648,17 +636,18 @@
         <v>10</v>
       </c>
       <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
+      <c r="D9" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="E9" s="4" t="n">
         <v>12000</v>
       </c>
-      <c r="F9" s="5" t="n"/>
     </row>
     <row r="10"/>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>COMO PREENCHER (meta mensal por produto):</t>
+          <t>COMO PREENCHER (meta mensal por produto) - TODOS os campos são obrigatórios:</t>
         </is>
       </c>
     </row>
@@ -672,66 +661,60 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>mes         -&gt; mês da meta (1 a 12). OPCIONAL: se em branco, usa o mês do seletor da tela. Com 'mes' preenchido, 1 arquivo cobre vários meses (revisões).</t>
+          <t>mes         -&gt; mês da meta (1 a 12). 1 arquivo cobre vários meses (revisões).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>territorio  -&gt; regional (valida contra o cadastro de Territórios). Em branco para Peças (nacional) e para Transgrain/Acessórios.</t>
+          <t>territorio  -&gt; regional (valida contra o cadastro de Territórios). Obrigatório, exceto para Peças (meta nacional).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>quantidade  -&gt; volume planejado no mês. OBRIGATÓRIO para tudo que não seja Peças</t>
+          <t>quantidade  -&gt; volume planejado no mês (Peças: opcional, a meta é em valor).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>valor       -&gt; valor planejado no mês em R$. Em branco, assume quantidade × FAT/un do cenário de planejamento. OBRIGATÓRIO só para Peças</t>
+          <t>valor       -&gt; valor planejado no mês em R$.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>MC1%         -&gt; MC1 %. Em branco, assume a do cenário de planejamento (premissas e impostos do FAT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18"/>
+          <t>Ao aplicar (Carga completa), só os MESES presentes no arquivo são substituídos; os ausentes ficam intactos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>O ANO e o CENÁRIO (Destino) são escolhidos na tela; só aparecem cenários sem formulário. Cenários com formulários usam o botão Importar do formulário FAT.</t>
+        </is>
+      </c>
+    </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Transgrain/Acessórios -&gt; território opcional; somam no card lateral do painel, por tipo. Peças usa a meta da coordenação Peças (Jenifer), em valor.</t>
+          <t>O sistema DERIVA: coordenação, responsável, linha de negócio, tipo, cultura.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Ao aplicar (Carga completa), só os MESES presentes no arquivo são substituídos; os ausentes ficam intactos.</t>
-        </is>
-      </c>
+      <c r="A20" s="6" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>O ANO e o CENÁRIO (Destino) são escolhidos na tela (seletor de período + Destino), não na planilha.</t>
-        </is>
-      </c>
+      <c r="A21" s="6" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>O sistema DERIVA: coordenação, responsável, linha de negócio, tipo, cultura.</t>
-        </is>
-      </c>
+      <c r="A22" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>